<commit_message>
Update Zenodo DOI and provenance note for v1.1.1
</commit_message>
<xml_diff>
--- a/data/Epistemic_Governor_Calibration_Matrix_TableA1.xlsx
+++ b/data/Epistemic_Governor_Calibration_Matrix_TableA1.xlsx
@@ -957,7 +957,7 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>LLM Phase 2 output — fabricated statistic; no source exists for this claim</t>
+          <t>LLM Phase 2 output — unsupported quantitative claim; no source support identified</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="17" t="inlineStr">
         <is>
-          <t>Note. Φ computed by PCR_Audit_Engine.py v6.0 using all-mpnet-base-v2 (Reimers &amp; Gurevych 2019; 768-D embeddings, mean pooling, cosine similarity). τ = .70 verification threshold. Source: PCR Master Execution Ledger, March 2026. Published dataset: Lindner JR, Clemons CA, McKibben JD (2026) AAD 7(2):109-124. doi:10.37433/aad.v7i2.637. N=80 (one incomplete response excluded from published study). PCR reference implementation used pre-publication aggregate (N=81; M=3.83, SD=1.09).</t>
+          <t>Note. Φ computed by PCR_Audit_Engine.py v6.0 using all-mpnet-base-v2 (Reimers &amp; Gurevych 2019; 768-D embeddings, mean pooling, cosine similarity). τ = .70 verification threshold. Source: PCR Master Execution Ledger, March 2026. Published dataset: Lindner JR, Clemons CA, McKibben JD (2026) AAD 7(2):109–124. doi:10.37433/aad.v7i2.637. The value N=81, M=3.83, SD=1.09 reflects a retained pre-publication aggregate from the Phase 1 dataset, later superseded by the published aggregate N=80, M=3.82, SD=1.07 after one incomplete response was excluded. This note clarifies provenance only and does not alter the manuscript's statistical reporting.</t>
         </is>
       </c>
     </row>

</xml_diff>